<commit_message>
ver - 1.6 changes
</commit_message>
<xml_diff>
--- a/Excel/Version 1/Bakery Products variants.xlsx
+++ b/Excel/Version 1/Bakery Products variants.xlsx
@@ -6069,7 +6069,7 @@
       </c>
       <c r="H2" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H2">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CKTUQLBETPJSJMY</v>
+        <v>BRZBFRUJBGRKASJ</v>
       </c>
       <c r="I2" s="2" t="s">
         <v>10</v>
@@ -6099,7 +6099,7 @@
       </c>
       <c r="H3" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H3">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>DFIWQHZBGZAADRV</v>
+        <v>EBYALANROCCDSYB</v>
       </c>
       <c r="I3" s="2" t="s">
         <v>10</v>
@@ -6129,7 +6129,7 @@
       </c>
       <c r="H4" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H4">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>RVZGLVUMMAUDIKG</v>
+        <v>FDBCZVCPVCGQQXW</v>
       </c>
       <c r="I4" s="2" t="s">
         <v>10</v>
@@ -6159,7 +6159,7 @@
       </c>
       <c r="H5" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H5">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>AOZWVRBQDICKJBI</v>
+        <v>CYRXYCUIQUHJRFY</v>
       </c>
       <c r="I5" s="2" t="s">
         <v>10</v>
@@ -6189,7 +6189,7 @@
       </c>
       <c r="H6" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H6">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>XQYSCNILWOAPROO</v>
+        <v>JUEBSSAVNFURPRW</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>10</v>
@@ -6219,7 +6219,7 @@
       </c>
       <c r="H7" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H7">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>IERXAXTNRUBKIUO</v>
+        <v>KUYCQLRYZRIPMAV</v>
       </c>
       <c r="I7" s="2" t="s">
         <v>10</v>
@@ -6249,7 +6249,7 @@
       </c>
       <c r="H8" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H8">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>RLAJPQFPMMEUFTQ</v>
+        <v>PDRTXYXKARSQJSA</v>
       </c>
       <c r="I8" s="2" t="s">
         <v>10</v>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="H9" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H9">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>AUEDAUMTHAKUKFT</v>
+        <v>GRTFYAPVTRLGHWT</v>
       </c>
       <c r="I9" s="2" t="s">
         <v>10</v>
@@ -6309,7 +6309,7 @@
       </c>
       <c r="H10" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H10">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CZURNIYFKJCZDML</v>
+        <v>GVJAQUFIGJITNHD</v>
       </c>
       <c r="I10" s="2" t="s">
         <v>10</v>
@@ -6339,7 +6339,7 @@
       </c>
       <c r="H11" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H11">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ZGVKAHXFYAUEYZH</v>
+        <v>VTYWYREONGTWUEH</v>
       </c>
       <c r="I11" s="2" t="s">
         <v>10</v>
@@ -6369,7 +6369,7 @@
       </c>
       <c r="H12" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H12">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>NAWPPBLGESQPZKF</v>
+        <v>NPICTVDNOWDJCWS</v>
       </c>
       <c r="I12" s="2" t="s">
         <v>10</v>
@@ -6399,7 +6399,7 @@
       </c>
       <c r="H13" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H13">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>RWMXNCVICBLWMSV</v>
+        <v>DBEKBIOJWJVXLBL</v>
       </c>
       <c r="I13" s="2" t="s">
         <v>10</v>
@@ -6429,7 +6429,7 @@
       </c>
       <c r="H14" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H14">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>LQLYFPHZXNYNDLT</v>
+        <v>APGLNLYZVYVHMGO</v>
       </c>
       <c r="I14" s="2" t="s">
         <v>10</v>
@@ -6459,7 +6459,7 @@
       </c>
       <c r="H15" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H15">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>BGAUIOEDPDXSCZM</v>
+        <v>NDAVYXNZCFIORPB</v>
       </c>
       <c r="I15" s="2" t="s">
         <v>10</v>
@@ -6489,7 +6489,7 @@
       </c>
       <c r="H16" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H16">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MMVARZXEZPXDULO</v>
+        <v>QHTTZTFDQLXUHNJ</v>
       </c>
       <c r="I16" s="2" t="s">
         <v>10</v>
@@ -6519,7 +6519,7 @@
       </c>
       <c r="H17" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H17">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>FMSHMMSISBGIYYK</v>
+        <v>GJSDMKXXEJUETFY</v>
       </c>
       <c r="I17" s="2" t="s">
         <v>10</v>
@@ -6549,7 +6549,7 @@
       </c>
       <c r="H18" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H18">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>PXGHSELSUODCSFU</v>
+        <v>YCEPRZMJPOBGCKR</v>
       </c>
       <c r="I18" s="2" t="s">
         <v>10</v>
@@ -6579,7 +6579,7 @@
       </c>
       <c r="H19" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H19">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>QUSVEILQKZNYRTV</v>
+        <v>WVWUPDNJOUWJSOC</v>
       </c>
       <c r="I19" s="2" t="s">
         <v>10</v>
@@ -6609,7 +6609,7 @@
       </c>
       <c r="H20" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H20">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>GVYPZWQGFMNMWIS</v>
+        <v>JBQJHTSYEYMQTLA</v>
       </c>
       <c r="I20" s="2" t="s">
         <v>10</v>
@@ -6639,7 +6639,7 @@
       </c>
       <c r="H21" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H21">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>TAPOMDKIVIERFQH</v>
+        <v>NULIMZANIOTWYXW</v>
       </c>
       <c r="I21" s="2" t="s">
         <v>10</v>
@@ -6669,7 +6669,7 @@
       </c>
       <c r="H22" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H22">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>FGWHLQNTMLFRJOJ</v>
+        <v>VLYXVUHEOXIUWBM</v>
       </c>
       <c r="I22" s="2" t="s">
         <v>10</v>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="H23" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H23">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MYOUQFAEKSMDEKJ</v>
+        <v>ACYJQYGURJOWCJC</v>
       </c>
       <c r="I23" s="2" t="s">
         <v>10</v>
@@ -6729,7 +6729,7 @@
       </c>
       <c r="H24" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H24">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>DRZKCWNETIPVUQA</v>
+        <v>NEEUCIUDHSRZGMW</v>
       </c>
       <c r="I24" s="2" t="s">
         <v>10</v>
@@ -6759,7 +6759,7 @@
       </c>
       <c r="H25" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H25">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>UXTMHNABZEGFJXE</v>
+        <v>HSZBMBSZPFEVCPB</v>
       </c>
       <c r="I25" s="2" t="s">
         <v>10</v>
@@ -6789,7 +6789,7 @@
       </c>
       <c r="H26" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H26">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>HIWXCRYVXHHQDGD</v>
+        <v>MIBRFSPGWWFMARR</v>
       </c>
       <c r="I26" s="2" t="s">
         <v>10</v>
@@ -6819,7 +6819,7 @@
       </c>
       <c r="H27" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H27">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>EBUERWCWNWWJRPD</v>
+        <v>USRUTHYKRDONWOU</v>
       </c>
       <c r="I27" s="2" t="s">
         <v>10</v>
@@ -6849,7 +6849,7 @@
       </c>
       <c r="H28" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H28">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>KIASOIWMUYIPNFX</v>
+        <v>EBLGRHIDTLKJDIU</v>
       </c>
       <c r="I28" s="2" t="s">
         <v>10</v>
@@ -6879,7 +6879,7 @@
       </c>
       <c r="H29" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H29">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ALUENAHDVBIQHBS</v>
+        <v>HSLEMMWKKMOMQYN</v>
       </c>
       <c r="I29" s="2" t="s">
         <v>10</v>
@@ -6909,7 +6909,7 @@
       </c>
       <c r="H30" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H30">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CPLFSVEOFKFDMPL</v>
+        <v>PLCAZAKJNBLFLZM</v>
       </c>
       <c r="I30" s="2" t="s">
         <v>10</v>
@@ -6939,7 +6939,7 @@
       </c>
       <c r="H31" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H31">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>JWIEYCUOPBVAQAY</v>
+        <v>LXRUPBRPJXYPDGF</v>
       </c>
       <c r="I31" s="2" t="s">
         <v>10</v>
@@ -6969,7 +6969,7 @@
       </c>
       <c r="H32" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H32">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>YJMKNVIOMNBALYG</v>
+        <v>GEYMAKXSLZCZYSR</v>
       </c>
       <c r="I32" s="2" t="s">
         <v>10</v>
@@ -6999,7 +6999,7 @@
       </c>
       <c r="H33" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H33">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>YIVPFXAIXVJMUNZ</v>
+        <v>ODRDUXKFZMQHHOP</v>
       </c>
       <c r="I33" s="2" t="s">
         <v>10</v>
@@ -7029,7 +7029,7 @@
       </c>
       <c r="H34" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H34">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>RTTDZQMUHGIPXGP</v>
+        <v>HPVICQRTGWHMRPZ</v>
       </c>
       <c r="I34" s="2" t="s">
         <v>10</v>
@@ -7059,7 +7059,7 @@
       </c>
       <c r="H35" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H35">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>NTLFCYTOZBOVKCC</v>
+        <v>KFEDERZXPTZFOCX</v>
       </c>
       <c r="I35" s="2" t="s">
         <v>10</v>
@@ -7089,7 +7089,7 @@
       </c>
       <c r="H36" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H36">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>DAIOCDSDJTPKUIP</v>
+        <v>TZQHCVTRRPIPHHK</v>
       </c>
       <c r="I36" s="2" t="s">
         <v>10</v>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="H37" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H37">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>WQRRZLWKRYYFYEG</v>
+        <v>GWOPINXEFARCARW</v>
       </c>
       <c r="I37" s="2" t="s">
         <v>10</v>
@@ -7149,7 +7149,7 @@
       </c>
       <c r="H38" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H38">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>GNHUGVNPUMINWUQ</v>
+        <v>WOGBRVKGJNGDLPN</v>
       </c>
       <c r="I38" s="2" t="s">
         <v>10</v>
@@ -7179,7 +7179,7 @@
       </c>
       <c r="H39" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H39">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ECNGFISUIBJYUXA</v>
+        <v>NAYHPBAVNBHDEJP</v>
       </c>
       <c r="I39" s="2" t="s">
         <v>10</v>
@@ -7209,7 +7209,7 @@
       </c>
       <c r="H40" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H40">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>VBZSMUQOAUCCSFF</v>
+        <v>FHQTOLLXPDVTQUU</v>
       </c>
       <c r="I40" s="2" t="s">
         <v>10</v>
@@ -7239,7 +7239,7 @@
       </c>
       <c r="H41" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H41">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>LBUIHHXCJQKGJPE</v>
+        <v>OCPZSKRPNRDUTGB</v>
       </c>
       <c r="I41" s="2" t="s">
         <v>10</v>
@@ -7269,7 +7269,7 @@
       </c>
       <c r="H42" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H42">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>BRVSSVFZINAPQRJ</v>
+        <v>WAZJALKGXBNPSZN</v>
       </c>
       <c r="I42" s="2" t="s">
         <v>10</v>
@@ -7299,7 +7299,7 @@
       </c>
       <c r="H43" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H43">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>IFINDQKGUNYFGCY</v>
+        <v>HUTSNCXLWRFXSNC</v>
       </c>
       <c r="I43" s="2" t="s">
         <v>10</v>
@@ -7329,7 +7329,7 @@
       </c>
       <c r="H44" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H44">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>FDATGVBJBHLUYGG</v>
+        <v>MJMYBFOCJTBBQOZ</v>
       </c>
       <c r="I44" s="2" t="s">
         <v>10</v>
@@ -7359,7 +7359,7 @@
       </c>
       <c r="H45" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H45">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>UCTDKEVJCCNZXKT</v>
+        <v>HWFWIVFEOKWZBWT</v>
       </c>
       <c r="I45" s="2" t="s">
         <v>10</v>
@@ -7389,7 +7389,7 @@
       </c>
       <c r="H46" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H46">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>WQHUXYBTSNPXVFD</v>
+        <v>IWIKUMKJCGLLLZV</v>
       </c>
       <c r="I46" s="2" t="s">
         <v>10</v>
@@ -7419,7 +7419,7 @@
       </c>
       <c r="H47" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H47">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>DQRHMRXTVLPQLEW</v>
+        <v>EUZZSQQYZTHUOEX</v>
       </c>
       <c r="I47" s="2" t="s">
         <v>10</v>
@@ -7449,7 +7449,7 @@
       </c>
       <c r="H48" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H48">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>QZYYLSJIRFUOVJM</v>
+        <v>CWEVGCPIDURWJBM</v>
       </c>
       <c r="I48" s="2" t="s">
         <v>10</v>
@@ -7479,7 +7479,7 @@
       </c>
       <c r="H49" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H49">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>NXDLLPYGCUKGKAY</v>
+        <v>PYISTVPZYJHMYYP</v>
       </c>
       <c r="I49" s="2" t="s">
         <v>10</v>
@@ -7509,7 +7509,7 @@
       </c>
       <c r="H50" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H50">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>OXQZLJQQTWZYHPF</v>
+        <v>SLPFJPVDPZEWVIE</v>
       </c>
       <c r="I50" s="2" t="s">
         <v>10</v>
@@ -7539,7 +7539,7 @@
       </c>
       <c r="H51" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H51">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>SDQAKWYPDJIQUNB</v>
+        <v>LAROJKNPFQVQQWJ</v>
       </c>
       <c r="I51" s="2" t="s">
         <v>10</v>
@@ -7569,7 +7569,7 @@
       </c>
       <c r="H52" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H52">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>XXNPWRJOGJAKZVU</v>
+        <v>CRTTASMSROEUGTP</v>
       </c>
       <c r="I52" s="2" t="s">
         <v>10</v>
@@ -7599,7 +7599,7 @@
       </c>
       <c r="H53" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H53">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>VLIPCOOWFPLXITR</v>
+        <v>XBRMAUKGBXVIMEO</v>
       </c>
       <c r="I53" s="2" t="s">
         <v>10</v>
@@ -7629,7 +7629,7 @@
       </c>
       <c r="H54" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H54">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>JWUJUJCREEUFVJY</v>
+        <v>JYFJFXZDSCHSCBN</v>
       </c>
       <c r="I54" s="2" t="s">
         <v>10</v>
@@ -7659,7 +7659,7 @@
       </c>
       <c r="H55" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H55">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MMWREMIRDPXDWNK</v>
+        <v>DDUIUHGHTALARJM</v>
       </c>
       <c r="I55" s="2" t="s">
         <v>10</v>
@@ -7689,7 +7689,7 @@
       </c>
       <c r="H56" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H56">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MKUNODCSABAWQPS</v>
+        <v>VIOSXDMLBROVYAG</v>
       </c>
       <c r="I56" s="2" t="s">
         <v>10</v>
@@ -7719,7 +7719,7 @@
       </c>
       <c r="H57" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H57">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>NJETSXUPGHFLMKU</v>
+        <v>GMUQYPCGKUPFDPT</v>
       </c>
       <c r="I57" s="2" t="s">
         <v>10</v>
@@ -7749,7 +7749,7 @@
       </c>
       <c r="H58" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H58">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MGPQQTNETKJWBUB</v>
+        <v>IIFFTBBMXXTFZAK</v>
       </c>
       <c r="I58" s="2" t="s">
         <v>10</v>
@@ -7779,7 +7779,7 @@
       </c>
       <c r="H59" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H59">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ZMJQQGHPGVXTIUQ</v>
+        <v>EZGDMZZRYXRJXGS</v>
       </c>
       <c r="I59" s="2" t="s">
         <v>10</v>
@@ -7809,7 +7809,7 @@
       </c>
       <c r="H60" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H60">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>EYDITZCSQUREVPZ</v>
+        <v>WHTRUFAQOFGSEPO</v>
       </c>
       <c r="I60" s="2" t="s">
         <v>10</v>
@@ -7839,7 +7839,7 @@
       </c>
       <c r="H61" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H61">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>VDQIRXTYEVJQOSO</v>
+        <v>KISMIGAKFEQGTNJ</v>
       </c>
       <c r="I61" s="2" t="s">
         <v>10</v>
@@ -7869,7 +7869,7 @@
       </c>
       <c r="H62" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H62">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MEEZKYNFABQHOVZ</v>
+        <v>JVXRMCBVXGKCFRU</v>
       </c>
       <c r="I62" s="2" t="s">
         <v>10</v>
@@ -7899,7 +7899,7 @@
       </c>
       <c r="H63" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H63">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CEWCZTQBBFNLPJX</v>
+        <v>PUSUHSWDEKBVLXM</v>
       </c>
       <c r="I63" s="2" t="s">
         <v>10</v>
@@ -7929,7 +7929,7 @@
       </c>
       <c r="H64" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H64">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>JZDUKMJHWFWQSPY</v>
+        <v>SVCPUSICYLEXTGJ</v>
       </c>
       <c r="I64" s="2" t="s">
         <v>10</v>
@@ -7959,7 +7959,7 @@
       </c>
       <c r="H65" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H65">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>WIDCHLJIPCPGDCJ</v>
+        <v>XBGLFMPYMVEIXBU</v>
       </c>
       <c r="I65" s="2" t="s">
         <v>10</v>
@@ -7989,7 +7989,7 @@
       </c>
       <c r="H66" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H66">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CWJMUSJXLZVKOEX</v>
+        <v>NUSPQHQTAEPOYJL</v>
       </c>
       <c r="I66" s="2" t="s">
         <v>10</v>
@@ -8019,7 +8019,7 @@
       </c>
       <c r="H67" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H67">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>VGWMVMBEBCEPEHN</v>
+        <v>LGENCCXGPAQUWMW</v>
       </c>
       <c r="I67" s="2" t="s">
         <v>10</v>
@@ -8049,7 +8049,7 @@
       </c>
       <c r="H68" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H68">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ZUXUDCXKGOQMIFB</v>
+        <v>PCVKIIWDJMQSYET</v>
       </c>
       <c r="I68" s="2" t="s">
         <v>10</v>
@@ -8079,7 +8079,7 @@
       </c>
       <c r="H69" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H69">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MYKHOTXMXCTOOJI</v>
+        <v>LJXCSBLQTPPAGBN</v>
       </c>
       <c r="I69" s="2" t="s">
         <v>10</v>
@@ -8109,7 +8109,7 @@
       </c>
       <c r="H70" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H70">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CKHYUYAXZVKFCZH</v>
+        <v>NICALLXXNAGOCWU</v>
       </c>
       <c r="I70" s="2" t="s">
         <v>10</v>
@@ -8139,7 +8139,7 @@
       </c>
       <c r="H71" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H71">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>CFUCXXOJGZKPWKR</v>
+        <v>QQGHCXIGDUMMUAF</v>
       </c>
       <c r="I71" s="2" t="s">
         <v>10</v>
@@ -8169,7 +8169,7 @@
       </c>
       <c r="H72" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H72">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>AJDQEFTDOGRNLVR</v>
+        <v>SIBPVOASEAIGHDK</v>
       </c>
       <c r="I72" s="2" t="s">
         <v>10</v>
@@ -8199,7 +8199,7 @@
       </c>
       <c r="H73" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H73">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>NZRPXUURMQROSYT</v>
+        <v>BIXTKMTFHRYYHCT</v>
       </c>
       <c r="I73" s="2" t="s">
         <v>10</v>
@@ -8229,7 +8229,7 @@
       </c>
       <c r="H74" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H74">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>BYANBTGZGKZNOQD</v>
+        <v>QNNLQXPSKFTLLZM</v>
       </c>
       <c r="I74" s="2" t="s">
         <v>10</v>
@@ -8259,7 +8259,7 @@
       </c>
       <c r="H75" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H75">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>FTFQAAXVRTMEMIL</v>
+        <v>ABYGUYPAFAXGNFX</v>
       </c>
       <c r="I75" s="2" t="s">
         <v>10</v>
@@ -8289,7 +8289,7 @@
       </c>
       <c r="H76" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H76">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MMTVRJZUQWQUECK</v>
+        <v>YBUVUYEIDVKBIPZ</v>
       </c>
       <c r="I76" s="2" t="s">
         <v>10</v>
@@ -8319,7 +8319,7 @@
       </c>
       <c r="H77" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H77">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MOGDRJZJHYLDIHN</v>
+        <v>MACZKQXWIOIQXKC</v>
       </c>
       <c r="I77" s="2" t="s">
         <v>10</v>
@@ -8349,7 +8349,7 @@
       </c>
       <c r="H78" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H78">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>JIRQELANUCPZSFI</v>
+        <v>GAKVYAPJLDWJRFL</v>
       </c>
       <c r="I78" s="2" t="s">
         <v>10</v>
@@ -8379,7 +8379,7 @@
       </c>
       <c r="H79" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H79">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>JAOKVDSDHAQASNX</v>
+        <v>MPCPQPVSAXJTARN</v>
       </c>
       <c r="I79" s="2" t="s">
         <v>10</v>
@@ -8409,7 +8409,7 @@
       </c>
       <c r="H80" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H80">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>TTPZSKUNLAAKHER</v>
+        <v>MOMEYZBUYABAPUZ</v>
       </c>
       <c r="I80" s="2" t="s">
         <v>10</v>
@@ -8439,7 +8439,7 @@
       </c>
       <c r="H81" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H81">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>JGYJADAVQMGGSKU</v>
+        <v>ZRQBXHWVWLEXBQF</v>
       </c>
       <c r="I81" s="2" t="s">
         <v>10</v>
@@ -8469,7 +8469,7 @@
       </c>
       <c r="H82" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H82">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>QMZEEVYWHBWVSEF</v>
+        <v>GQRUTMQEJXWPVZV</v>
       </c>
       <c r="I82" s="2" t="s">
         <v>10</v>
@@ -8499,7 +8499,7 @@
       </c>
       <c r="H83" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H83">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>OLRFHABULDUTRON</v>
+        <v>XDLEIAXTUREPIRO</v>
       </c>
       <c r="I83" s="2" t="s">
         <v>10</v>
@@ -8529,7 +8529,7 @@
       </c>
       <c r="H84" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H84">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>OZACIUZCJOOLKAQ</v>
+        <v>FDFNSMELZFDVVBM</v>
       </c>
       <c r="I84" s="2" t="s">
         <v>10</v>
@@ -8559,7 +8559,7 @@
       </c>
       <c r="H85" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H85">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>RPLVQXMNYORTXGM</v>
+        <v>SHXIYMPJIJBTUFJ</v>
       </c>
       <c r="I85" s="2" t="s">
         <v>10</v>
@@ -8589,7 +8589,7 @@
       </c>
       <c r="H86" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H86">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>UTBOKERIBWTOFHI</v>
+        <v>BLHIXVSJJIWUCCA</v>
       </c>
       <c r="I86" s="2" t="s">
         <v>10</v>
@@ -8619,7 +8619,7 @@
       </c>
       <c r="H87" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H87">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>OEQKDKCWGZXGKOQ</v>
+        <v>ZDQREKAHTZGSKLV</v>
       </c>
       <c r="I87" s="2" t="s">
         <v>10</v>
@@ -8649,7 +8649,7 @@
       </c>
       <c r="H88" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H88">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>FISEQMFYCKMFXRU</v>
+        <v>OEREXCYGCFSCWGY</v>
       </c>
       <c r="I88" s="2" t="s">
         <v>10</v>
@@ -8679,7 +8679,7 @@
       </c>
       <c r="H89" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H89">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>UYPCCJZVJVSRUSY</v>
+        <v>NPQQSSBVATZOJOA</v>
       </c>
       <c r="I89" s="2" t="s">
         <v>10</v>
@@ -8709,7 +8709,7 @@
       </c>
       <c r="H90" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H90">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>EZFIJPIOLWDSFWI</v>
+        <v>QGXNZUBZDMZLZBX</v>
       </c>
       <c r="I90" s="2" t="s">
         <v>10</v>
@@ -8739,7 +8739,7 @@
       </c>
       <c r="H91" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H91">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>NEXDMYUBSPOOEQU</v>
+        <v>UWYJJPOGBBEWZKT</v>
       </c>
       <c r="I91" s="2" t="s">
         <v>10</v>
@@ -8769,7 +8769,7 @@
       </c>
       <c r="H92" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H92">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ELPOTNKFFHFUQDM</v>
+        <v>VVQBSPTYVTLPBTW</v>
       </c>
       <c r="I92" s="2" t="s">
         <v>10</v>
@@ -8799,7 +8799,7 @@
       </c>
       <c r="H93" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H93">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>SWECYUQFETXYFJX</v>
+        <v>RLALYXMZWPOHTYD</v>
       </c>
       <c r="I93" s="2" t="s">
         <v>10</v>
@@ -8829,7 +8829,7 @@
       </c>
       <c r="H94" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H94">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>MCWKSDGIEDPQUME</v>
+        <v>YCAHGDVWDVSFLPH</v>
       </c>
       <c r="I94" s="2" t="s">
         <v>10</v>
@@ -8859,7 +8859,7 @@
       </c>
       <c r="H95" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H95">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>QWFPIVSQYCQPZIL</v>
+        <v>MXVWGZMBSUIIFUS</v>
       </c>
       <c r="I95" s="2" t="s">
         <v>10</v>
@@ -8889,7 +8889,7 @@
       </c>
       <c r="H96" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H96">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>BZDWGHUKFXKZMXB</v>
+        <v>ZMESPPLCDJRXKWY</v>
       </c>
       <c r="I96" s="2" t="s">
         <v>10</v>
@@ -8919,7 +8919,7 @@
       </c>
       <c r="H97" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H97">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>TQRXWUYGMBQMTGT</v>
+        <v>EAJRFOFFMLFWYSL</v>
       </c>
       <c r="I97" s="2" t="s">
         <v>10</v>
@@ -8949,7 +8949,7 @@
       </c>
       <c r="H98" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H98">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ZBKLXYBWTMWOZKS</v>
+        <v>HPTVPNIPLFILQBM</v>
       </c>
       <c r="I98" s="2" t="s">
         <v>10</v>
@@ -8979,7 +8979,7 @@
       </c>
       <c r="H99" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H99">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>YUHBUQRQPEJPVGZ</v>
+        <v>FCBRAJMNEKUNICD</v>
       </c>
       <c r="I99" s="2" t="s">
         <v>10</v>
@@ -9009,7 +9009,7 @@
       </c>
       <c r="H100" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H100">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>LYIKVYTFUITVCHL</v>
+        <v>OSAPGYLXQLNZSRJ</v>
       </c>
       <c r="I100" s="2" t="s">
         <v>10</v>
@@ -9039,7 +9039,7 @@
       </c>
       <c r="H101" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H101">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>COUHXKXQQUQVWTZ</v>
+        <v>VHDXGFNUNYAMRCG</v>
       </c>
       <c r="I101" s="2" t="s">
         <v>10</v>
@@ -9069,7 +9069,7 @@
       </c>
       <c r="H102" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H102">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>XVVYUJDRPAWSDCP</v>
+        <v>VXLMALRGYDVEZQJ</v>
       </c>
       <c r="I102" s="2" t="s">
         <v>10</v>
@@ -9099,7 +9099,7 @@
       </c>
       <c r="H103" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H103">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>LQYBZXEQPPGTBNF</v>
+        <v>TBXOHYWLDURWKNV</v>
       </c>
       <c r="I103" s="2" t="s">
         <v>10</v>
@@ -9129,7 +9129,7 @@
       </c>
       <c r="H104" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H104">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>GNHCXOXLLGQGIWA</v>
+        <v>TBVIEWQBULSQHLJ</v>
       </c>
       <c r="I104" s="2" t="s">
         <v>10</v>
@@ -9159,7 +9159,7 @@
       </c>
       <c r="H105" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H105">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>UMGNUDPELTMFTVS</v>
+        <v>QJRKDQOKDJIJJCU</v>
       </c>
       <c r="I105" s="2" t="s">
         <v>10</v>
@@ -9189,7 +9189,7 @@
       </c>
       <c r="H106" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H106">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>GSVRLTVXQZHPZUN</v>
+        <v>TJUABIZFFBFUZAF</v>
       </c>
       <c r="I106" s="2" t="s">
         <v>10</v>
@@ -9219,7 +9219,7 @@
       </c>
       <c r="H107" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H107">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>XWCERBWRQJLYYOU</v>
+        <v>NFVFLICMWSIODZE</v>
       </c>
       <c r="I107" s="2" t="s">
         <v>10</v>
@@ -9249,7 +9249,7 @@
       </c>
       <c r="H108" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H108">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>XPGPGBQGSXVTXYR</v>
+        <v>ASCDMXPIWWFNLQV</v>
       </c>
       <c r="I108" s="2" t="s">
         <v>10</v>
@@ -9279,7 +9279,7 @@
       </c>
       <c r="H109" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H109">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>LAYNOINFTHUQXRO</v>
+        <v>CNWMGQWOHCGYDAX</v>
       </c>
       <c r="I109" s="2" t="s">
         <v>10</v>
@@ -9309,7 +9309,7 @@
       </c>
       <c r="H110" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H110">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>YDVHIIGMUOWBZDZ</v>
+        <v>XAZPWSPTBLVXNLS</v>
       </c>
       <c r="I110" s="2" t="s">
         <v>10</v>
@@ -9339,7 +9339,7 @@
       </c>
       <c r="H111" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H111">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>IYIVKZHFTVQGJQX</v>
+        <v>NQGORXNBHUNDNXM</v>
       </c>
       <c r="I111" s="2" t="s">
         <v>10</v>
@@ -9369,7 +9369,7 @@
       </c>
       <c r="H112" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H112">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>UZQRLXGYHSJAYQG</v>
+        <v>OKMMOPNBZNHPXDR</v>
       </c>
       <c r="I112" s="2" t="s">
         <v>10</v>
@@ -9399,7 +9399,7 @@
       </c>
       <c r="H113" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H113">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>ESJXNJDORZYZOXG</v>
+        <v>UXGASBUHMOTTGTH</v>
       </c>
       <c r="I113" s="2" t="s">
         <v>10</v>
@@ -9429,7 +9429,7 @@
       </c>
       <c r="H114" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H114">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>AIXRQQYFPJWAOHZ</v>
+        <v>YUNNPYNMUAZDXOL</v>
       </c>
       <c r="I114" s="2" t="s">
         <v>10</v>
@@ -9459,7 +9459,7 @@
       </c>
       <c r="H115" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H115">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>RETYOSIASQSHPLX</v>
+        <v>XLXISPVTZKFPFTI</v>
       </c>
       <c r="I115" s="2" t="s">
         <v>10</v>
@@ -9489,7 +9489,7 @@
       </c>
       <c r="H116" s="6" t="str" cm="1">
         <f ca="1" t="array" ref="H116">_xlfn.TEXTJOIN("",TRUE,CHAR(RANDBETWEEN(65,90+0*_xlfn.SEQUENCE(15))))</f>
-        <v>INOVTLEEXZBLZQO</v>
+        <v>EIERWKAWRTQYMKD</v>
       </c>
       <c r="I116" s="2" t="s">
         <v>10</v>
@@ -9508,7 +9508,6 @@
     <row r="118" ht="15.6" spans="2:9">
       <c r="B118" s="7"/>
       <c r="C118" s="7"/>
-      <c r="D118" s="2"/>
       <c r="E118" s="8"/>
       <c r="F118" s="8"/>
       <c r="G118" s="7"/>
@@ -9518,8 +9517,6 @@
     <row r="119" ht="15.6" spans="2:9">
       <c r="B119" s="7"/>
       <c r="C119" s="7"/>
-      <c r="D119" s="2"/>
-      <c r="E119" s="2"/>
       <c r="F119" s="8"/>
       <c r="G119" s="7"/>
       <c r="H119" s="6"/>
@@ -9558,7 +9555,6 @@
     <row r="123" ht="15.6" spans="2:9">
       <c r="B123" s="7"/>
       <c r="C123" s="7"/>
-      <c r="D123" s="2"/>
       <c r="E123" s="8"/>
       <c r="F123" s="8"/>
       <c r="G123" s="7"/>
@@ -9588,8 +9584,6 @@
     <row r="126" ht="15.6" spans="2:9">
       <c r="B126" s="7"/>
       <c r="C126" s="7"/>
-      <c r="D126" s="2"/>
-      <c r="E126" s="2"/>
       <c r="F126" s="8"/>
       <c r="G126" s="7"/>
       <c r="H126" s="6"/>
@@ -9639,7 +9633,6 @@
       <c r="B131" s="7"/>
       <c r="C131" s="7"/>
       <c r="D131" s="8"/>
-      <c r="E131" s="2"/>
       <c r="F131" s="8"/>
       <c r="G131" s="7"/>
       <c r="H131" s="6"/>
@@ -9658,7 +9651,6 @@
     <row r="133" ht="15.6" spans="2:9">
       <c r="B133" s="7"/>
       <c r="C133" s="7"/>
-      <c r="D133" s="2"/>
       <c r="E133" s="8"/>
       <c r="F133" s="8"/>
       <c r="G133" s="7"/>
@@ -9668,8 +9660,6 @@
     <row r="134" ht="15.6" spans="2:9">
       <c r="B134" s="7"/>
       <c r="C134" s="7"/>
-      <c r="D134" s="2"/>
-      <c r="E134" s="2"/>
       <c r="F134" s="8"/>
       <c r="G134" s="7"/>
       <c r="H134" s="6"/>
@@ -9708,7 +9698,6 @@
     <row r="138" ht="15.6" spans="2:9">
       <c r="B138" s="7"/>
       <c r="C138" s="7"/>
-      <c r="D138" s="2"/>
       <c r="E138" s="8"/>
       <c r="F138" s="8"/>
       <c r="G138" s="7"/>
@@ -9738,8 +9727,6 @@
     <row r="141" ht="15.6" spans="2:9">
       <c r="B141" s="7"/>
       <c r="C141" s="7"/>
-      <c r="D141" s="2"/>
-      <c r="E141" s="2"/>
       <c r="F141" s="8"/>
       <c r="G141" s="7"/>
       <c r="H141" s="6"/>
@@ -9808,7 +9795,6 @@
     <row r="148" ht="15.6" spans="2:9">
       <c r="B148" s="7"/>
       <c r="C148" s="7"/>
-      <c r="D148" s="2"/>
       <c r="E148" s="8"/>
       <c r="F148" s="8"/>
       <c r="G148" s="7"/>
@@ -9838,8 +9824,6 @@
     <row r="151" ht="15.6" spans="2:9">
       <c r="B151" s="7"/>
       <c r="C151" s="7"/>
-      <c r="D151" s="2"/>
-      <c r="E151" s="2"/>
       <c r="F151" s="8"/>
       <c r="G151" s="7"/>
       <c r="H151" s="6"/>
@@ -9889,7 +9873,6 @@
       <c r="B156" s="7"/>
       <c r="C156" s="7"/>
       <c r="D156" s="8"/>
-      <c r="E156" s="2"/>
       <c r="F156" s="8"/>
       <c r="G156" s="7"/>
       <c r="H156" s="6"/>
@@ -9908,7 +9891,6 @@
     <row r="158" ht="15.6" spans="2:9">
       <c r="B158" s="7"/>
       <c r="C158" s="7"/>
-      <c r="D158" s="2"/>
       <c r="E158" s="8"/>
       <c r="F158" s="8"/>
       <c r="G158" s="7"/>
@@ -9918,8 +9900,6 @@
     <row r="159" ht="15.6" spans="2:9">
       <c r="B159" s="7"/>
       <c r="C159" s="7"/>
-      <c r="D159" s="2"/>
-      <c r="E159" s="2"/>
       <c r="F159" s="8"/>
       <c r="G159" s="7"/>
       <c r="H159" s="6"/>
@@ -9958,7 +9938,6 @@
     <row r="163" ht="15.6" spans="2:9">
       <c r="B163" s="7"/>
       <c r="C163" s="7"/>
-      <c r="D163" s="2"/>
       <c r="E163" s="8"/>
       <c r="F163" s="8"/>
       <c r="G163" s="7"/>
@@ -9988,8 +9967,6 @@
     <row r="166" ht="15.6" spans="2:9">
       <c r="B166" s="7"/>
       <c r="C166" s="7"/>
-      <c r="D166" s="2"/>
-      <c r="E166" s="2"/>
       <c r="F166" s="8"/>
       <c r="G166" s="7"/>
       <c r="H166" s="6"/>
@@ -10039,7 +10016,6 @@
       <c r="B171" s="7"/>
       <c r="C171" s="7"/>
       <c r="D171" s="8"/>
-      <c r="E171" s="2"/>
       <c r="F171" s="8"/>
       <c r="G171" s="7"/>
       <c r="H171" s="6"/>
@@ -10078,7 +10054,6 @@
     <row r="175" ht="15.6" spans="2:9">
       <c r="B175" s="7"/>
       <c r="C175" s="7"/>
-      <c r="D175" s="2"/>
       <c r="E175" s="8"/>
       <c r="F175" s="8"/>
       <c r="G175" s="7"/>
@@ -10108,8 +10083,6 @@
     <row r="178" ht="15.6" spans="2:9">
       <c r="B178" s="7"/>
       <c r="C178" s="7"/>
-      <c r="D178" s="2"/>
-      <c r="E178" s="2"/>
       <c r="F178" s="8"/>
       <c r="G178" s="7"/>
       <c r="H178" s="6"/>
@@ -10159,7 +10132,6 @@
       <c r="B183" s="7"/>
       <c r="C183" s="7"/>
       <c r="D183" s="8"/>
-      <c r="E183" s="2"/>
       <c r="F183" s="8"/>
       <c r="G183" s="7"/>
       <c r="H183" s="6"/>
@@ -10178,7 +10150,6 @@
     <row r="185" ht="15.6" spans="2:9">
       <c r="B185" s="7"/>
       <c r="C185" s="7"/>
-      <c r="D185" s="2"/>
       <c r="E185" s="8"/>
       <c r="F185" s="8"/>
       <c r="G185" s="7"/>
@@ -10188,8 +10159,6 @@
     <row r="186" ht="15.6" spans="2:9">
       <c r="B186" s="7"/>
       <c r="C186" s="7"/>
-      <c r="D186" s="2"/>
-      <c r="E186" s="2"/>
       <c r="F186" s="8"/>
       <c r="G186" s="7"/>
       <c r="H186" s="6"/>

</xml_diff>